<commit_message>
Improved 2114 pio and associated timings. Fixed a log flush bug that was DOSing the main task loop under heavy logging load.
</commit_message>
<xml_diff>
--- a/firmware/timings/2114-100.xlsx
+++ b/firmware/timings/2114-100.xlsx
@@ -8,34 +8,35 @@
   </sheets>
   <definedNames>
     <definedName name="tWC_start">Timings!$K$4</definedName>
-    <definedName name="tCO_end">Timings!$K$22</definedName>
+    <definedName name="tCO_end">Timings!$K$26</definedName>
     <definedName name="tRC_start">Timings!$K$4</definedName>
-    <definedName name="tDH_start">Timings!$K$14</definedName>
-    <definedName name="tOTD_start">Timings!$K$25</definedName>
-    <definedName name="tCO_start">Timings!$K$19</definedName>
+    <definedName name="tCO_start">Timings!$K$22</definedName>
     <definedName name="branch">Timings!$K$7</definedName>
-    <definedName name="tOTD_end">Timings!$K$30</definedName>
     <definedName name="tRC_end">Timings!$K$30</definedName>
     <definedName name="tW_end">Timings!$K$14</definedName>
-    <definedName name="tDH_end">Timings!$K$17</definedName>
     <definedName name="tDW_end">Timings!$K$14</definedName>
+    <definedName name="tA">Timings!$B$22</definedName>
+    <definedName name="tA_start">Timings!$K$6</definedName>
+    <definedName name="tCO">Timings!$B$21</definedName>
+    <definedName name="tA_sub_tCO_end">Timings!$K$21</definedName>
     <definedName name="tW_start">Timings!$K$9</definedName>
     <definedName name="tDW_start">Timings!$K$6</definedName>
-    <definedName name="tolerance">Timings!$B$30</definedName>
+    <definedName name="tolerance">Timings!$B$28</definedName>
     <definedName name="tWC_end">Timings!$K$17</definedName>
+    <definedName name="tA_end">Timings!$K$26</definedName>
     <definedName name="inst_ns">Timings!$I$2</definedName>
   </definedNames>
   <calcPr/>
   <extLst>
     <ext uri="GoogleSheetsCustomDataVersion2">
-      <go:sheetsCustomData xmlns:go="http://customooxmlschemas.google.com/" r:id="rId6" roundtripDataChecksum="8BlZARZ68vVYxDZWeEHSeosyXe3zO0FcMouS65Rh88Q="/>
+      <go:sheetsCustomData xmlns:go="http://customooxmlschemas.google.com/" r:id="rId6" roundtripDataChecksum="+8wULw/kt9rCioUKB4RcHRFh9jJ8UP7HmX4WPFbhhWg="/>
     </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="86" uniqueCount="78">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="97" uniqueCount="91">
   <si>
     <t>#</t>
   </si>
@@ -91,19 +92,28 @@
     <t>pull block</t>
   </si>
   <si>
-    <t>Get the next command. Let's start tRC/tWC loop here.</t>
+    <t>Get the next command. Start tWC and tRC.</t>
+  </si>
+  <si>
+    <t>tW 1</t>
   </si>
   <si>
     <t>out x, 1</t>
   </si>
   <si>
-    <t>Get first bit - which tells us if we are in write mode.</t>
+    <t>Get write mode bit.</t>
+  </si>
+  <si>
+    <t>tW 2</t>
   </si>
   <si>
     <t>out pins, 17</t>
   </si>
   <si>
-    <t>Load address, data, and CMD_ALL_OFF. Start of tDW.</t>
+    <t xml:space="preserve">Load address, data, and CMD_ALL_OFF. Start of tDW. Start of tRC, tA, tWC, tW. </t>
+  </si>
+  <si>
+    <t>tWC 1</t>
   </si>
   <si>
     <t>jmp !x read_branch</t>
@@ -112,13 +122,19 @@
     <t>Skip write if not in write mode</t>
   </si>
   <si>
+    <t>tWC 2</t>
+  </si>
+  <si>
     <t>write_branch:</t>
   </si>
   <si>
     <t>mov pindirs, ~NULL</t>
   </si>
   <si>
-    <t>All pins are outputs to ram.</t>
+    <t>All pins act as outputs to ram.</t>
+  </si>
+  <si>
+    <t>tA-tCO 1</t>
   </si>
   <si>
     <t>set pins, CMD_ALL_ON</t>
@@ -127,10 +143,16 @@
     <t xml:space="preserve">Lower CS and WE. Start of tW. </t>
   </si>
   <si>
+    <t>tA-tCO 2</t>
+  </si>
+  <si>
     <t>nop [1]</t>
   </si>
   <si>
     <t>tW delay1.</t>
+  </si>
+  <si>
+    <t>tA-tCO 3</t>
   </si>
   <si>
     <t>nop [2]</t>
@@ -139,10 +161,16 @@
     <t>tW delay2.</t>
   </si>
   <si>
+    <t>tCO 1</t>
+  </si>
+  <si>
     <t>in NULL, 32</t>
   </si>
   <si>
     <t>Need to let C code know we are finished!</t>
+  </si>
+  <si>
+    <t>tCO 2</t>
   </si>
   <si>
     <t>push noblock</t>
@@ -151,16 +179,19 @@
     <t>Send ISR to input FIFO.</t>
   </si>
   <si>
+    <t>tCO 3</t>
+  </si>
+  <si>
     <t>set pins, CMD_ALL_OFF</t>
   </si>
   <si>
-    <t>End of write pulse. tW, tDW must be met. Start of tDH.</t>
+    <t>End of write pulse. tW, tDW must be met.</t>
   </si>
   <si>
     <t>nop [3]</t>
   </si>
   <si>
-    <t>Write cycle recovery time 1.</t>
+    <t>tWC delay 1</t>
   </si>
   <si>
     <t>Datasheet Timings</t>
@@ -175,13 +206,16 @@
     <t>nop [4]</t>
   </si>
   <si>
+    <t>tWC delay 2</t>
+  </si>
+  <si>
     <t>tW</t>
   </si>
   <si>
     <t>jmp begin</t>
   </si>
   <si>
-    <t>tDH, tWC must be met.</t>
+    <t>tWC must be met.</t>
   </si>
   <si>
     <t>tDW</t>
@@ -199,37 +233,64 @@
     <t>tWC</t>
   </si>
   <si>
-    <t>set pins, CMD_CS_ON</t>
+    <t>nop [5]</t>
   </si>
   <si>
-    <t>Lower CS only. Start of tCO.</t>
+    <t>tA-tCO delay 1.</t>
+  </si>
+  <si>
+    <t>tA-tCO</t>
+  </si>
+  <si>
+    <t>nop [6]</t>
+  </si>
+  <si>
+    <t>tA-tCO delay 2.</t>
   </si>
   <si>
     <t>tCO</t>
   </si>
   <si>
-    <t>nop[5]</t>
+    <t>nop [7]</t>
+  </si>
+  <si>
+    <t>tA-tCO delay 3.</t>
+  </si>
+  <si>
+    <t>tA</t>
+  </si>
+  <si>
+    <t>set pins, CMD_CS_ON</t>
+  </si>
+  <si>
+    <t>Lower CS only. tA-tCO must be met. Start of tCO.</t>
+  </si>
+  <si>
+    <t>tRC</t>
+  </si>
+  <si>
+    <t>nop [8]</t>
   </si>
   <si>
     <t>tCO delay 1.</t>
   </si>
   <si>
-    <t>tOTD</t>
-  </si>
-  <si>
-    <t>nop[6]</t>
+    <t>nop [9]</t>
   </si>
   <si>
     <t>tCO delay 2.</t>
   </si>
   <si>
-    <t>tRC</t>
+    <t>nop [10]</t>
+  </si>
+  <si>
+    <t>tCO delay 3.</t>
   </si>
   <si>
     <t>in pins, 17</t>
   </si>
   <si>
-    <t>Sample pins into ISR. tCO mst be met.</t>
+    <t>Sample the data into the ISR. tA and tCO mst be met.</t>
   </si>
   <si>
     <t>in NULL, 15</t>
@@ -238,34 +299,13 @@
     <t>Shift pins right so they start at LSB of ISR.</t>
   </si>
   <si>
-    <t>Deselect the data. Start of tOTD.</t>
-  </si>
-  <si>
-    <t>nop [7]</t>
-  </si>
-  <si>
-    <t>Read cycle recovery time 1.</t>
-  </si>
-  <si>
-    <t>nop [8]</t>
-  </si>
-  <si>
-    <t>Read cycle recovery time 2.</t>
-  </si>
-  <si>
-    <t>nop [9]</t>
-  </si>
-  <si>
-    <t>Read cycle recovery time 3.</t>
-  </si>
-  <si>
-    <t>nop [10]</t>
-  </si>
-  <si>
     <t>Tolerance %</t>
   </si>
   <si>
-    <t>tOTD, tRC must be met.</t>
+    <t>Deselect the data.</t>
+  </si>
+  <si>
+    <t>tRC must be met.</t>
   </si>
   <si>
     <t>Where data sheets differ, the tightest value across all available sheets has been used.</t>
@@ -484,7 +524,7 @@
   <cellStyleXfs count="1">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
   </cellStyleXfs>
-  <cellXfs count="46">
+  <cellXfs count="45">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
@@ -588,16 +628,13 @@
     </xf>
     <xf borderId="4" fillId="0" fontId="6" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
     <xf borderId="6" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment shrinkToFit="0" vertical="center" wrapText="0"/>
+    </xf>
+    <xf borderId="6" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="center" wrapText="0"/>
     </xf>
-    <xf borderId="7" fillId="0" fontId="2" numFmtId="1" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
+    <xf borderId="2" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="right" shrinkToFit="0" vertical="center" wrapText="0"/>
-    </xf>
-    <xf borderId="7" fillId="0" fontId="2" numFmtId="164" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
-      <alignment horizontal="right" shrinkToFit="0" vertical="center" wrapText="0"/>
-    </xf>
-    <xf borderId="2" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment horizontal="right" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="0"/>
     </xf>
     <xf borderId="10" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="right" shrinkToFit="0" vertical="center" wrapText="0"/>
@@ -4892,7 +4929,8 @@
   <cols>
     <col customWidth="1" min="1" max="1" width="11.13"/>
     <col customWidth="1" min="2" max="2" width="8.63"/>
-    <col customWidth="1" min="3" max="4" width="10.0"/>
+    <col customWidth="1" min="3" max="3" width="8.88"/>
+    <col customWidth="1" min="4" max="4" width="10.0"/>
     <col customWidth="1" min="5" max="6" width="3.13"/>
     <col customWidth="1" min="7" max="7" width="17.25"/>
     <col customWidth="1" min="8" max="8" width="23.75"/>
@@ -5004,15 +5042,17 @@
         <v>1.0</v>
       </c>
       <c r="B5" s="31">
-        <v>16.0</v>
-      </c>
-      <c r="C5" s="26"/>
+        <v>15.0</v>
+      </c>
+      <c r="C5" s="27" t="s">
+        <v>19</v>
+      </c>
       <c r="D5" s="26"/>
       <c r="E5" s="26"/>
       <c r="F5" s="26"/>
       <c r="G5" s="27"/>
       <c r="H5" s="28" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="I5" s="28">
         <v>0.0</v>
@@ -5026,7 +5066,7 @@
         <v>6.6666</v>
       </c>
       <c r="L5" s="28" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
     </row>
     <row r="6" ht="15.75" customHeight="1">
@@ -5036,13 +5076,15 @@
       <c r="B6" s="25">
         <v>0.0</v>
       </c>
-      <c r="C6" s="26"/>
+      <c r="C6" s="27" t="s">
+        <v>22</v>
+      </c>
       <c r="D6" s="26"/>
       <c r="E6" s="26"/>
       <c r="F6" s="26"/>
       <c r="G6" s="27"/>
       <c r="H6" s="28" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="I6" s="28">
         <v>0.0</v>
@@ -5056,23 +5098,25 @@
         <v>9.9999</v>
       </c>
       <c r="L6" s="28" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
     </row>
     <row r="7" ht="15.75" customHeight="1">
       <c r="A7" s="30">
         <v>3.0</v>
       </c>
-      <c r="B7" s="25">
+      <c r="B7" s="31">
         <v>0.0</v>
       </c>
-      <c r="C7" s="26"/>
+      <c r="C7" s="27" t="s">
+        <v>25</v>
+      </c>
       <c r="D7" s="26"/>
       <c r="E7" s="26"/>
       <c r="F7" s="26"/>
       <c r="G7" s="27"/>
       <c r="H7" s="28" t="s">
-        <v>23</v>
+        <v>26</v>
       </c>
       <c r="I7" s="28">
         <v>0.0</v>
@@ -5086,25 +5130,27 @@
         <v>13.3332</v>
       </c>
       <c r="L7" s="28" t="s">
-        <v>24</v>
+        <v>27</v>
       </c>
     </row>
     <row r="8" ht="15.75" customHeight="1">
       <c r="A8" s="30">
         <v>4.0</v>
       </c>
-      <c r="B8" s="31">
+      <c r="B8" s="25">
         <v>0.0</v>
       </c>
-      <c r="C8" s="26"/>
+      <c r="C8" s="27" t="s">
+        <v>28</v>
+      </c>
       <c r="D8" s="26"/>
       <c r="E8" s="26"/>
       <c r="F8" s="26"/>
       <c r="G8" s="27" t="s">
-        <v>25</v>
+        <v>29</v>
       </c>
       <c r="H8" s="28" t="s">
-        <v>26</v>
+        <v>30</v>
       </c>
       <c r="I8" s="28">
         <v>0.0</v>
@@ -5118,7 +5164,7 @@
         <v>16.6665</v>
       </c>
       <c r="L8" s="28" t="s">
-        <v>27</v>
+        <v>31</v>
       </c>
     </row>
     <row r="9" ht="15.75" customHeight="1">
@@ -5126,15 +5172,17 @@
         <v>5.0</v>
       </c>
       <c r="B9" s="31">
-        <v>17.0</v>
-      </c>
-      <c r="C9" s="26"/>
+        <v>3.0</v>
+      </c>
+      <c r="C9" s="27" t="s">
+        <v>32</v>
+      </c>
       <c r="D9" s="26"/>
       <c r="E9" s="26"/>
       <c r="F9" s="26"/>
       <c r="G9" s="27"/>
       <c r="H9" s="28" t="s">
-        <v>28</v>
+        <v>33</v>
       </c>
       <c r="I9" s="28">
         <v>0.0</v>
@@ -5148,7 +5196,7 @@
         <v>19.9998</v>
       </c>
       <c r="L9" s="28" t="s">
-        <v>29</v>
+        <v>34</v>
       </c>
     </row>
     <row r="10" ht="15.75" customHeight="1">
@@ -5158,13 +5206,15 @@
       <c r="B10" s="25">
         <v>0.0</v>
       </c>
-      <c r="C10" s="26"/>
+      <c r="C10" s="27" t="s">
+        <v>35</v>
+      </c>
       <c r="D10" s="26"/>
       <c r="E10" s="26"/>
       <c r="F10" s="26"/>
       <c r="G10" s="27"/>
       <c r="H10" s="28" t="s">
-        <v>30</v>
+        <v>36</v>
       </c>
       <c r="I10" s="28">
         <v>1.0</v>
@@ -5175,50 +5225,54 @@
       </c>
       <c r="K10" s="29">
         <f>J10+(OFFSET($B$4,$I10,0)+1)*inst_ns</f>
-        <v>76.6659</v>
+        <v>73.3326</v>
       </c>
       <c r="L10" s="28" t="s">
-        <v>31</v>
+        <v>37</v>
       </c>
     </row>
     <row r="11" ht="15.75" customHeight="1">
       <c r="A11" s="30">
         <v>7.0</v>
       </c>
-      <c r="B11" s="31">
-        <v>4.0</v>
-      </c>
-      <c r="C11" s="26"/>
+      <c r="B11" s="25">
+        <v>0.0</v>
+      </c>
+      <c r="C11" s="27" t="s">
+        <v>38</v>
+      </c>
       <c r="D11" s="26"/>
       <c r="E11" s="26"/>
       <c r="F11" s="26"/>
       <c r="G11" s="27"/>
       <c r="H11" s="28" t="s">
-        <v>32</v>
+        <v>39</v>
       </c>
       <c r="I11" s="28">
         <v>2.0</v>
       </c>
       <c r="J11" s="32">
         <f t="shared" si="2"/>
-        <v>76.6659</v>
+        <v>73.3326</v>
       </c>
       <c r="K11" s="29">
         <f>J11+(OFFSET($B$4,$I11,0)+1)*inst_ns</f>
-        <v>79.9992</v>
+        <v>76.6659</v>
       </c>
       <c r="L11" s="28" t="s">
-        <v>33</v>
+        <v>40</v>
       </c>
     </row>
     <row r="12" ht="15.75" customHeight="1">
       <c r="A12" s="30">
         <v>8.0</v>
       </c>
-      <c r="B12" s="25">
-        <v>0.0</v>
-      </c>
-      <c r="C12" s="26"/>
+      <c r="B12" s="31">
+        <v>15.0</v>
+      </c>
+      <c r="C12" s="27" t="s">
+        <v>41</v>
+      </c>
       <c r="D12" s="26" t="s">
         <v>5</v>
       </c>
@@ -5226,21 +5280,21 @@
       <c r="F12" s="26"/>
       <c r="G12" s="27"/>
       <c r="H12" s="28" t="s">
-        <v>34</v>
+        <v>42</v>
       </c>
       <c r="I12" s="28">
         <v>0.0</v>
       </c>
       <c r="J12" s="29">
         <f t="shared" si="2"/>
-        <v>79.9992</v>
+        <v>76.6659</v>
       </c>
       <c r="K12" s="29">
         <f>J12+(OFFSET($B$4,$I12,0)+1)*inst_ns</f>
-        <v>83.3325</v>
+        <v>79.9992</v>
       </c>
       <c r="L12" s="28" t="s">
-        <v>35</v>
+        <v>43</v>
       </c>
     </row>
     <row r="13" ht="15.75" customHeight="1">
@@ -5249,26 +5303,29 @@
       </c>
       <c r="B13" s="25">
         <v>0.0</v>
+      </c>
+      <c r="C13" s="27" t="s">
+        <v>44</v>
       </c>
       <c r="E13" s="19"/>
       <c r="F13" s="19"/>
       <c r="G13" s="27"/>
       <c r="H13" s="28" t="s">
-        <v>36</v>
+        <v>45</v>
       </c>
       <c r="I13" s="28">
         <v>0.0</v>
       </c>
       <c r="J13" s="32">
         <f t="shared" si="2"/>
-        <v>83.3325</v>
+        <v>79.9992</v>
       </c>
       <c r="K13" s="29">
         <f>J13+(OFFSET($B$4,$I13,0)+1)*inst_ns</f>
-        <v>86.6658</v>
+        <v>83.3325</v>
       </c>
       <c r="L13" s="28" t="s">
-        <v>37</v>
+        <v>46</v>
       </c>
     </row>
     <row r="14" ht="15.75" customHeight="1">
@@ -5277,26 +5334,29 @@
       </c>
       <c r="B14" s="25">
         <v>0.0</v>
+      </c>
+      <c r="C14" s="27" t="s">
+        <v>47</v>
       </c>
       <c r="E14" s="19"/>
       <c r="F14" s="19"/>
       <c r="G14" s="27"/>
       <c r="H14" s="28" t="s">
-        <v>38</v>
+        <v>48</v>
       </c>
       <c r="I14" s="28">
         <v>0.0</v>
       </c>
       <c r="J14" s="29">
         <f t="shared" si="2"/>
-        <v>86.6658</v>
+        <v>83.3325</v>
       </c>
       <c r="K14" s="29">
         <f>J14+(OFFSET($B$4,$I14,0)+1)*inst_ns</f>
-        <v>89.9991</v>
+        <v>86.6658</v>
       </c>
       <c r="L14" s="28" t="s">
-        <v>39</v>
+        <v>49</v>
       </c>
     </row>
     <row r="15" ht="15.75" customHeight="1">
@@ -5304,113 +5364,113 @@
       <c r="F15" s="19"/>
       <c r="G15" s="27"/>
       <c r="H15" s="28" t="s">
-        <v>40</v>
+        <v>50</v>
       </c>
       <c r="I15" s="28">
         <v>3.0</v>
       </c>
       <c r="J15" s="29">
         <f t="shared" si="2"/>
-        <v>89.9991</v>
+        <v>86.6658</v>
       </c>
       <c r="K15" s="29">
         <f>J15+(OFFSET($B$4,$I15,0)+1)*inst_ns</f>
-        <v>93.3324</v>
+        <v>89.9991</v>
       </c>
       <c r="L15" s="28" t="s">
-        <v>41</v>
+        <v>51</v>
       </c>
     </row>
     <row r="16" ht="15.75" customHeight="1">
       <c r="A16" s="9" t="s">
-        <v>42</v>
+        <v>52</v>
       </c>
       <c r="B16" s="10"/>
       <c r="C16" s="16" t="s">
-        <v>43</v>
+        <v>53</v>
       </c>
       <c r="D16" s="16" t="s">
-        <v>44</v>
+        <v>54</v>
       </c>
       <c r="E16" s="19"/>
       <c r="F16" s="19"/>
       <c r="G16" s="27"/>
       <c r="H16" s="28" t="s">
-        <v>45</v>
+        <v>55</v>
       </c>
       <c r="I16" s="28">
         <v>4.0</v>
       </c>
       <c r="J16" s="29">
         <f t="shared" si="2"/>
-        <v>93.3324</v>
+        <v>89.9991</v>
       </c>
       <c r="K16" s="29">
         <f>J16+(OFFSET($B$4,$I16,0)+1)*inst_ns</f>
-        <v>96.6657</v>
+        <v>93.3324</v>
       </c>
       <c r="L16" s="28" t="s">
-        <v>41</v>
+        <v>56</v>
       </c>
     </row>
     <row r="17" ht="15.75" customHeight="1">
       <c r="A17" s="30" t="s">
-        <v>46</v>
+        <v>57</v>
       </c>
       <c r="B17" s="25">
         <v>75.0</v>
       </c>
       <c r="C17" s="33">
         <f>B17 + (B17 * tolerance/100)</f>
-        <v>69.75</v>
+        <v>67.5</v>
       </c>
       <c r="D17" s="34">
         <f>ROUND(tW_end - tW_start,1)</f>
-        <v>70</v>
+        <v>66.7</v>
       </c>
       <c r="E17" s="19"/>
       <c r="F17" s="19"/>
       <c r="G17" s="35"/>
       <c r="H17" s="28" t="s">
-        <v>47</v>
+        <v>58</v>
       </c>
       <c r="I17" s="28">
         <v>0.0</v>
       </c>
       <c r="J17" s="32">
         <f t="shared" si="2"/>
-        <v>96.6657</v>
+        <v>93.3324</v>
       </c>
       <c r="K17" s="29">
         <f>J17+(OFFSET($B$4,$I17,0)+1)*inst_ns</f>
-        <v>99.999</v>
+        <v>96.6657</v>
       </c>
       <c r="L17" s="28" t="s">
-        <v>48</v>
+        <v>59</v>
       </c>
     </row>
     <row r="18" ht="15.75" customHeight="1">
       <c r="A18" s="30" t="s">
-        <v>49</v>
+        <v>60</v>
       </c>
       <c r="B18" s="25">
         <v>70.0</v>
       </c>
       <c r="C18" s="33">
         <f>B18 + (B18 * tolerance/100)</f>
-        <v>65.1</v>
+        <v>63</v>
       </c>
       <c r="D18" s="34">
         <f>ROUND(tDW_end - tDW_start,1)</f>
-        <v>80</v>
+        <v>76.7</v>
       </c>
       <c r="E18" s="19"/>
       <c r="F18" s="19"/>
       <c r="G18" s="27" t="s">
-        <v>50</v>
+        <v>61</v>
       </c>
       <c r="H18" s="28" t="s">
-        <v>51</v>
+        <v>62</v>
       </c>
       <c r="I18" s="28">
         <v>0.0</v>
@@ -5424,177 +5484,185 @@
         <v>16.6665</v>
       </c>
       <c r="L18" s="28" t="s">
-        <v>52</v>
+        <v>63</v>
       </c>
     </row>
     <row r="19" ht="15.75" customHeight="1">
       <c r="A19" s="30" t="s">
-        <v>53</v>
+        <v>64</v>
       </c>
       <c r="B19" s="31">
         <v>100.0</v>
       </c>
       <c r="C19" s="33">
         <f>B19 + (B19 * tolerance/100)</f>
-        <v>93</v>
+        <v>90</v>
       </c>
       <c r="D19" s="34">
         <f>ROUND(tWC_end - tWC_start, 1)</f>
-        <v>96.7</v>
+        <v>93.3</v>
       </c>
       <c r="E19" s="19"/>
       <c r="F19" s="19"/>
       <c r="G19" s="27"/>
       <c r="H19" s="28" t="s">
-        <v>54</v>
+        <v>65</v>
       </c>
       <c r="I19" s="28">
-        <v>0.0</v>
-      </c>
-      <c r="J19" s="29">
+        <v>5.0</v>
+      </c>
+      <c r="J19" s="32">
         <f t="shared" ref="J19:J30" si="3">K18</f>
         <v>16.6665</v>
       </c>
       <c r="K19" s="29">
         <f>J19+(OFFSET($B$4,$I19,0)+1)*inst_ns</f>
-        <v>19.9998</v>
+        <v>29.9997</v>
       </c>
       <c r="L19" s="28" t="s">
-        <v>55</v>
+        <v>66</v>
       </c>
     </row>
     <row r="20" ht="15.75" customHeight="1">
       <c r="A20" s="30" t="s">
-        <v>56</v>
-      </c>
-      <c r="B20" s="25">
-        <v>70.0</v>
+        <v>67</v>
+      </c>
+      <c r="B20" s="36">
+        <f>tA-tCO</f>
+        <v>30</v>
       </c>
       <c r="C20" s="33">
         <f>B20 + (B20 * tolerance/100)</f>
-        <v>65.1</v>
+        <v>27</v>
       </c>
       <c r="D20" s="34">
-        <f>ROUND(tCO_end - tCO_start,1)</f>
-        <v>66.7</v>
+        <f>ROUND(tA_sub_tCO_end - tA_start,1)</f>
+        <v>26.7</v>
       </c>
       <c r="E20" s="19"/>
       <c r="F20" s="19"/>
       <c r="G20" s="27"/>
       <c r="H20" s="28" t="s">
-        <v>57</v>
+        <v>68</v>
       </c>
       <c r="I20" s="28">
-        <v>5.0</v>
+        <v>6.0</v>
       </c>
       <c r="J20" s="32">
         <f t="shared" si="3"/>
-        <v>19.9998</v>
+        <v>29.9997</v>
       </c>
       <c r="K20" s="29">
         <f>J20+(OFFSET($B$4,$I20,0)+1)*inst_ns</f>
-        <v>79.9992</v>
+        <v>33.333</v>
       </c>
       <c r="L20" s="28" t="s">
-        <v>58</v>
-      </c>
-    </row>
-    <row r="21" ht="15.75" customHeight="1">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="21">
       <c r="A21" s="30" t="s">
-        <v>59</v>
-      </c>
-      <c r="B21" s="36">
-        <v>30.0</v>
+        <v>70</v>
+      </c>
+      <c r="B21" s="25">
+        <v>70.0</v>
       </c>
       <c r="C21" s="33">
         <f>B21 + (B21 * tolerance/100)</f>
-        <v>27.9</v>
+        <v>63</v>
       </c>
       <c r="D21" s="34">
-        <f>ROUND(tOTD_end - tOTD_start,1)</f>
-        <v>30</v>
-      </c>
-      <c r="E21" s="19"/>
-      <c r="F21" s="19"/>
-      <c r="G21" s="27"/>
+        <f>ROUND(tCO_end - tCO_start,1)</f>
+        <v>63.3</v>
+      </c>
+      <c r="G21" s="35"/>
       <c r="H21" s="28" t="s">
-        <v>60</v>
+        <v>71</v>
       </c>
       <c r="I21" s="28">
-        <v>6.0</v>
-      </c>
-      <c r="J21" s="32">
+        <v>7.0</v>
+      </c>
+      <c r="J21" s="29">
         <f t="shared" si="3"/>
-        <v>79.9992</v>
+        <v>33.333</v>
       </c>
       <c r="K21" s="29">
         <f>J21+(OFFSET($B$4,$I21,0)+1)*inst_ns</f>
-        <v>83.3325</v>
+        <v>36.6663</v>
       </c>
       <c r="L21" s="28" t="s">
-        <v>61</v>
+        <v>72</v>
       </c>
     </row>
     <row r="22" ht="15.75" customHeight="1">
       <c r="A22" s="30" t="s">
-        <v>62</v>
-      </c>
-      <c r="B22" s="31">
+        <v>73</v>
+      </c>
+      <c r="B22" s="37">
         <v>100.0</v>
       </c>
       <c r="C22" s="33">
         <f>B22 + (B22 * tolerance/100)</f>
-        <v>93</v>
+        <v>90</v>
       </c>
       <c r="D22" s="34">
-        <f>ROUND(tRC_end - tRC_start, 1)</f>
-        <v>123.3</v>
+        <f>ROUND(tA_end - tA_start, 1)</f>
+        <v>93.3</v>
       </c>
       <c r="E22" s="19"/>
       <c r="F22" s="19"/>
-      <c r="G22" s="35"/>
-      <c r="H22" s="35" t="s">
-        <v>63</v>
+      <c r="G22" s="27"/>
+      <c r="H22" s="28" t="s">
+        <v>74</v>
       </c>
       <c r="I22" s="28">
         <v>0.0</v>
       </c>
       <c r="J22" s="29">
         <f t="shared" si="3"/>
-        <v>83.3325</v>
+        <v>36.6663</v>
       </c>
       <c r="K22" s="29">
         <f>J22+(OFFSET($B$4,$I22,0)+1)*inst_ns</f>
-        <v>86.6658</v>
+        <v>39.9996</v>
       </c>
       <c r="L22" s="28" t="s">
-        <v>64</v>
+        <v>75</v>
       </c>
     </row>
     <row r="23" ht="15.75" customHeight="1">
-      <c r="A23" s="30"/>
-      <c r="B23" s="25"/>
-      <c r="C23" s="33"/>
-      <c r="D23" s="34"/>
+      <c r="A23" s="30" t="s">
+        <v>76</v>
+      </c>
+      <c r="B23" s="31">
+        <v>100.0</v>
+      </c>
+      <c r="C23" s="33">
+        <f>B23 + (B23 * tolerance/100)</f>
+        <v>90</v>
+      </c>
+      <c r="D23" s="34">
+        <f>ROUND(tRC_end - tRC_start, 1)</f>
+        <v>113.3</v>
+      </c>
       <c r="E23" s="19"/>
       <c r="F23" s="19"/>
-      <c r="G23" s="27"/>
       <c r="H23" s="28" t="s">
-        <v>65</v>
+        <v>77</v>
       </c>
       <c r="I23" s="28">
-        <v>0.0</v>
+        <v>8.0</v>
       </c>
       <c r="J23" s="29">
         <f t="shared" si="3"/>
-        <v>86.6658</v>
+        <v>39.9996</v>
       </c>
       <c r="K23" s="29">
         <f>J23+(OFFSET($B$4,$I23,0)+1)*inst_ns</f>
-        <v>89.9991</v>
+        <v>93.3324</v>
       </c>
       <c r="L23" s="28" t="s">
-        <v>66</v>
+        <v>78</v>
       </c>
     </row>
     <row r="24" ht="15.75" customHeight="1">
@@ -5604,23 +5672,23 @@
       <c r="D24" s="34"/>
       <c r="E24" s="19"/>
       <c r="F24" s="19"/>
-      <c r="G24" s="27"/>
+      <c r="G24" s="35"/>
       <c r="H24" s="28" t="s">
-        <v>36</v>
+        <v>79</v>
       </c>
       <c r="I24" s="28">
-        <v>0.0</v>
-      </c>
-      <c r="J24" s="32">
+        <v>9.0</v>
+      </c>
+      <c r="J24" s="29">
         <f t="shared" si="3"/>
-        <v>89.9991</v>
+        <v>93.3324</v>
       </c>
       <c r="K24" s="29">
         <f>J24+(OFFSET($B$4,$I24,0)+1)*inst_ns</f>
-        <v>93.3324</v>
+        <v>96.6657</v>
       </c>
       <c r="L24" s="28" t="s">
-        <v>37</v>
+        <v>80</v>
       </c>
     </row>
     <row r="25">
@@ -5632,21 +5700,21 @@
       <c r="F25" s="19"/>
       <c r="G25" s="35"/>
       <c r="H25" s="28" t="s">
-        <v>38</v>
+        <v>81</v>
       </c>
       <c r="I25" s="28">
-        <v>0.0</v>
+        <v>10.0</v>
       </c>
       <c r="J25" s="29">
         <f t="shared" si="3"/>
-        <v>93.3324</v>
+        <v>96.6657</v>
       </c>
       <c r="K25" s="29">
         <f>J25+(OFFSET($B$4,$I25,0)+1)*inst_ns</f>
-        <v>96.6657</v>
+        <v>99.999</v>
       </c>
       <c r="L25" s="28" t="s">
-        <v>67</v>
+        <v>82</v>
       </c>
     </row>
     <row r="26" ht="15.75" customHeight="1">
@@ -5657,22 +5725,22 @@
       <c r="E26" s="19"/>
       <c r="F26" s="19"/>
       <c r="G26" s="35"/>
-      <c r="H26" s="28" t="s">
-        <v>68</v>
+      <c r="H26" s="35" t="s">
+        <v>83</v>
       </c>
       <c r="I26" s="28">
-        <v>7.0</v>
+        <v>0.0</v>
       </c>
       <c r="J26" s="29">
         <f t="shared" si="3"/>
-        <v>96.6657</v>
+        <v>99.999</v>
       </c>
       <c r="K26" s="29">
         <f>J26+(OFFSET($B$4,$I26,0)+1)*inst_ns</f>
-        <v>113.3322</v>
+        <v>103.3323</v>
       </c>
       <c r="L26" s="28" t="s">
-        <v>69</v>
+        <v>84</v>
       </c>
     </row>
     <row r="27" ht="15.75" customHeight="1">
@@ -5682,116 +5750,108 @@
       <c r="D27" s="34"/>
       <c r="E27" s="19"/>
       <c r="F27" s="19"/>
-      <c r="G27" s="35"/>
+      <c r="G27" s="27"/>
       <c r="H27" s="28" t="s">
-        <v>70</v>
+        <v>85</v>
       </c>
       <c r="I27" s="28">
-        <v>8.0</v>
+        <v>0.0</v>
       </c>
       <c r="J27" s="29">
         <f t="shared" si="3"/>
-        <v>113.3322</v>
+        <v>103.3323</v>
       </c>
       <c r="K27" s="29">
         <f>J27+(OFFSET($B$4,$I27,0)+1)*inst_ns</f>
-        <v>116.6655</v>
+        <v>106.6656</v>
       </c>
       <c r="L27" s="28" t="s">
-        <v>71</v>
+        <v>86</v>
       </c>
     </row>
     <row r="28" ht="15.75" customHeight="1">
-      <c r="A28" s="30"/>
-      <c r="B28" s="25"/>
-      <c r="C28" s="33"/>
-      <c r="D28" s="34"/>
+      <c r="A28" s="30" t="s">
+        <v>87</v>
+      </c>
+      <c r="B28" s="38">
+        <v>-10.0</v>
+      </c>
+      <c r="C28" s="39"/>
+      <c r="D28" s="40"/>
       <c r="E28" s="19"/>
       <c r="F28" s="19"/>
-      <c r="G28" s="35"/>
+      <c r="G28" s="27"/>
       <c r="H28" s="28" t="s">
-        <v>72</v>
+        <v>45</v>
       </c>
       <c r="I28" s="28">
-        <v>9.0</v>
-      </c>
-      <c r="J28" s="29">
+        <v>0.0</v>
+      </c>
+      <c r="J28" s="32">
         <f t="shared" si="3"/>
-        <v>116.6655</v>
+        <v>106.6656</v>
       </c>
       <c r="K28" s="29">
         <f>J28+(OFFSET($B$4,$I28,0)+1)*inst_ns</f>
-        <v>119.9988</v>
+        <v>109.9989</v>
       </c>
       <c r="L28" s="28" t="s">
-        <v>73</v>
+        <v>46</v>
       </c>
     </row>
     <row r="29" ht="15.75" customHeight="1">
-      <c r="A29" s="30"/>
-      <c r="B29" s="25"/>
-      <c r="C29" s="37"/>
-      <c r="D29" s="38"/>
       <c r="E29" s="19"/>
       <c r="F29" s="19"/>
       <c r="G29" s="35"/>
       <c r="H29" s="28" t="s">
-        <v>74</v>
+        <v>48</v>
       </c>
       <c r="I29" s="28">
-        <v>10.0</v>
+        <v>0.0</v>
       </c>
       <c r="J29" s="29">
         <f t="shared" si="3"/>
-        <v>119.9988</v>
+        <v>109.9989</v>
       </c>
       <c r="K29" s="29">
         <f>J29+(OFFSET($B$4,$I29,0)+1)*inst_ns</f>
-        <v>123.3321</v>
+        <v>113.3322</v>
       </c>
       <c r="L29" s="28" t="s">
-        <v>73</v>
+        <v>88</v>
       </c>
     </row>
     <row r="30" ht="15.75" customHeight="1">
-      <c r="A30" s="30" t="s">
-        <v>75</v>
-      </c>
-      <c r="B30" s="39">
-        <v>-7.0</v>
-      </c>
-      <c r="C30" s="40"/>
-      <c r="D30" s="41"/>
       <c r="E30" s="19"/>
       <c r="F30" s="19"/>
       <c r="G30" s="35"/>
       <c r="H30" s="28" t="s">
-        <v>47</v>
+        <v>58</v>
       </c>
       <c r="I30" s="28">
         <v>0.0</v>
       </c>
       <c r="J30" s="32">
         <f t="shared" si="3"/>
-        <v>123.3321</v>
+        <v>113.3322</v>
       </c>
       <c r="K30" s="29">
         <f>J30+(OFFSET($B$4,$I30,0)+1)*inst_ns</f>
-        <v>126.6654</v>
+        <v>116.6655</v>
       </c>
       <c r="L30" s="28" t="s">
-        <v>76</v>
+        <v>89</v>
       </c>
     </row>
     <row r="31" ht="15.75" customHeight="1">
       <c r="E31" s="26"/>
       <c r="F31" s="26"/>
-      <c r="G31" s="35"/>
-      <c r="H31" s="35"/>
-      <c r="I31" s="35"/>
-      <c r="J31" s="35"/>
-      <c r="K31" s="35"/>
-      <c r="L31" s="35"/>
+      <c r="G31" s="27"/>
+      <c r="H31" s="28"/>
+      <c r="I31" s="28"/>
+      <c r="J31" s="41"/>
+      <c r="K31" s="28"/>
+      <c r="L31" s="28"/>
     </row>
     <row r="32">
       <c r="A32" s="19"/>
@@ -5800,28 +5860,16 @@
       <c r="D32" s="19"/>
       <c r="E32" s="26"/>
       <c r="F32" s="26"/>
-      <c r="G32" s="27"/>
-      <c r="H32" s="28"/>
-      <c r="I32" s="28"/>
-      <c r="J32" s="42"/>
-      <c r="K32" s="28"/>
-      <c r="L32" s="28"/>
     </row>
     <row r="33">
-      <c r="A33" s="43" t="s">
-        <v>77</v>
-      </c>
-      <c r="B33" s="44"/>
-      <c r="C33" s="44"/>
-      <c r="D33" s="45"/>
+      <c r="A33" s="42" t="s">
+        <v>90</v>
+      </c>
+      <c r="B33" s="43"/>
+      <c r="C33" s="43"/>
+      <c r="D33" s="44"/>
       <c r="E33" s="7"/>
       <c r="F33" s="7"/>
-      <c r="G33" s="7"/>
-      <c r="H33" s="7"/>
-      <c r="I33" s="7"/>
-      <c r="J33" s="7"/>
-      <c r="K33" s="7"/>
-      <c r="L33" s="7"/>
     </row>
     <row r="34" ht="15.75" customHeight="1">
       <c r="A34" s="6"/>
@@ -5830,12 +5878,6 @@
       <c r="D34" s="6"/>
       <c r="E34" s="6"/>
       <c r="F34" s="6"/>
-      <c r="G34" s="6"/>
-      <c r="H34" s="6"/>
-      <c r="I34" s="6"/>
-      <c r="J34" s="6"/>
-      <c r="K34" s="6"/>
-      <c r="L34" s="6"/>
     </row>
     <row r="35" ht="15.75" customHeight="1">
       <c r="A35" s="6"/>
@@ -5844,12 +5886,6 @@
       <c r="D35" s="6"/>
       <c r="E35" s="6"/>
       <c r="F35" s="6"/>
-      <c r="G35" s="6"/>
-      <c r="H35" s="6"/>
-      <c r="I35" s="6"/>
-      <c r="J35" s="6"/>
-      <c r="K35" s="6"/>
-      <c r="L35" s="6"/>
     </row>
     <row r="36" ht="15.75" customHeight="1">
       <c r="A36" s="6"/>
@@ -5858,12 +5894,6 @@
       <c r="D36" s="6"/>
       <c r="E36" s="6"/>
       <c r="F36" s="6"/>
-      <c r="G36" s="6"/>
-      <c r="H36" s="6"/>
-      <c r="I36" s="6"/>
-      <c r="J36" s="6"/>
-      <c r="K36" s="6"/>
-      <c r="L36" s="6"/>
     </row>
     <row r="37" ht="15.75" customHeight="1">
       <c r="A37" s="6"/>
@@ -19378,59 +19408,44 @@
       <formula>D17&lt;C17</formula>
     </cfRule>
   </conditionalFormatting>
+  <conditionalFormatting sqref="D26">
+    <cfRule type="expression" dxfId="0" priority="3">
+      <formula>D26&lt;C26</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="D27">
+    <cfRule type="expression" dxfId="0" priority="4">
+      <formula>D27&lt;C27</formula>
+    </cfRule>
+  </conditionalFormatting>
   <conditionalFormatting sqref="D24">
-    <cfRule type="expression" dxfId="0" priority="3">
+    <cfRule type="expression" dxfId="0" priority="5">
       <formula>D24&lt;C24</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="D23">
-    <cfRule type="expression" dxfId="0" priority="4">
-      <formula>D23&lt;C23</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="D27">
-    <cfRule type="expression" dxfId="0" priority="5">
-      <formula>D27&lt;C27</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="D28">
-    <cfRule type="expression" dxfId="0" priority="6">
-      <formula>D28&lt;C28</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="D29">
-    <cfRule type="expression" dxfId="1" priority="7">
-      <formula>D29&lt;C29</formula>
-    </cfRule>
-  </conditionalFormatting>
   <conditionalFormatting sqref="D25">
-    <cfRule type="expression" dxfId="0" priority="8">
+    <cfRule type="expression" dxfId="1" priority="6">
       <formula>D25&lt;C25</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="D26">
-    <cfRule type="expression" dxfId="1" priority="9">
-      <formula>D26&lt;C26</formula>
-    </cfRule>
-  </conditionalFormatting>
   <conditionalFormatting sqref="D19">
-    <cfRule type="expression" dxfId="0" priority="10">
+    <cfRule type="expression" dxfId="0" priority="7">
       <formula>D19&lt;C19</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="D20">
-    <cfRule type="expression" dxfId="0" priority="11">
+  <conditionalFormatting sqref="D21">
+    <cfRule type="expression" dxfId="0" priority="8">
+      <formula>D21&lt;C21</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="D20 D22">
+    <cfRule type="expression" dxfId="0" priority="9">
       <formula>D20&lt;C20</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="D21">
-    <cfRule type="expression" dxfId="0" priority="12">
-      <formula>D21&lt;C21</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="D22">
-    <cfRule type="expression" dxfId="0" priority="13">
-      <formula>D22&lt;C22</formula>
+  <conditionalFormatting sqref="D23">
+    <cfRule type="expression" dxfId="0" priority="10">
+      <formula>D23&lt;C23</formula>
     </cfRule>
   </conditionalFormatting>
   <printOptions/>

</xml_diff>